<commit_message>
Merged reading for extraction and risk of bias in both guides and workbook READMEs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRD7etKqYN8v2bbXeeLMRW
</commit_message>
<xml_diff>
--- a/search/rob/rob_R1_blank.xlsx
+++ b/search/rob/rob_R1_blank.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -495,113 +495,120 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>• 每篇报告一行；每个条目选 Yes（满足）/ No / Unclear。条目文字见下方，是对 Murad 等 2018 和协议第 15 节的转述，请对照原文核对。</t>
+          <t>• 和正式提取合并阅读：每篇全文只读一遍，同一遍里填提取表和这份偏倚风险表（作者 2026-10-25 同意）。两份表仍各自独立，由两人分别填。</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>• 每篇报告一行；每个条目选 Yes（满足）/ No / Unclear。条目文字见下方，是对 Murad 等 2018 和协议第 15 节的转述，请对照原文核对。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
           <t>• 不算总分。adequate 列是公式：持续时间（exposure）、结局（outcome）、报告充分性（reporting）三项都是 Yes 才是 Yes；三项都填了而有一项不是 Yes 为 No；没填完为空。Unclear 按未满足算（这是 Claude 的读法，待确认）。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>• 按这篇报告里用于主要问题的患者整体来评价；一篇里不同患者情况不同时，按多数或最关键的患者判断，并在 note 里写明。</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>• 按这篇报告里用于主要问题的患者整体来评价；一篇里不同患者情况不同时，按多数或最关键的患者判断，并在 note 里写明。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>• 挑战-再挑战、剂量-反应两项不适用，已省略（协议第 15 节）。本院 5 例不评价。</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>条目</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>• selection（Selection）：Do the patients represent the whole experience of the investigators (centre), or is the selection method stated, so that other similar patients are unlikely to have been left out?</t>
         </is>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>• selection（Selection）：Do the patients represent the whole experience of the investigators (centre), or is the selection method stated, so that other similar patients are unlikely to have been left out?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>• exposure（Ascertainment of exposure）：Are the timing of symptom onset and of operation stated precisely enough to give the duration of the index episode?</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>• outcome（Ascertainment of outcome）：Is splenic viability at operation stated, with its basis (operative findings or histology)?</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>• alternative（Alternative explanations）：Were other explanations for the outcome considered or ruled out (for example, the spleen removed for a technical reason, or a pre-existing splenic disease)?</t>
         </is>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>• alternative（Alternative explanations）：Were other explanations for the outcome considered or ruled out (for example, the spleen removed for a technical reason, or a pre-existing splenic disease)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>• followup（Adequacy of follow-up）：Was follow-up long enough for the outcomes of interest (splenic status, recurrence) to occur, and is it reported?</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>• reporting（Sufficiency of reporting）：Are the patients described in enough detail for others to use the information in their own practice?</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>做完以后</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>• 各自另存带日期的副本。两人都做完后运行 `python3 -I tools/compare_rob.py compare 文件R1.xlsx 文件R2.xlsx --out DIR`，得到分歧清单；讨论，讨论不了的交杨俊；统一后的结果写入 rob.csv（报告编号、adequate），供敏感性分析 5 使用。</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>• 评价员是谁协议第 15 节只写了'两位评价员'；这里按提取员（舒俊、卞红强）安排，这是提议，待确认。</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>没有验证的事</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>• 没有在 Excel 或 WPS 里打开过；下拉列表、公式和版面是否正常没有验证。</t>
         </is>

</xml_diff>